<commit_message>
Integracion de filtros de tiempo al modulo de productos
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_exportacion_productos.xlsx
+++ b/public/templates/plantilla_exportacion_productos.xlsx
@@ -2,19 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\plantillas general\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DEAA051-2033-40A9-A026-691A093601F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259C8898-D7AC-40D4-BE7E-8C8A7EDFC5B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B8A71F7A-89C4-4348-A586-7AFA6FFC93FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{29730ABD-B3A1-4C07-BD99-22D4B675851D}"/>
   </bookViews>
   <sheets>
-    <sheet name="InvFisicoValoradoConsolidado" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$L$10</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -31,28 +34,52 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>Nombre de la empresa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIT: </t>
+  </si>
+  <si>
+    <t>Casa Matriz:</t>
+  </si>
+  <si>
+    <t>La Paz - Bolivia</t>
+  </si>
   <si>
     <t>COD. ITEM</t>
   </si>
   <si>
+    <t>DESCRIPCION</t>
+  </si>
+  <si>
     <t>UNIDAD</t>
   </si>
   <si>
+    <t>P/U</t>
+  </si>
+  <si>
+    <t>DEL (FECHA DE INICIO) AL (FECHA FINAL)</t>
+  </si>
+  <si>
+    <t>(Expresado en Bolivianos)</t>
+  </si>
+  <si>
     <t>NOMBRE</t>
   </si>
   <si>
     <t>MARCA</t>
   </si>
   <si>
-    <t>DESCRIPCIÓN</t>
-  </si>
-  <si>
     <t>METODO DE INVENTARIO</t>
   </si>
   <si>
@@ -65,56 +92,100 @@
     <t>STOCK</t>
   </si>
   <si>
-    <t>P/U</t>
-  </si>
-  <si>
-    <t>PRECIO DE VENTA</t>
+    <t>PRECIO VENTA</t>
+  </si>
+  <si>
+    <t>CATALOGO DE PRODUCTOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <u/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="5"/>
-      <name val="Calibri"/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -124,42 +195,141 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -167,39 +337,69 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -220,9 +420,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -230,39 +430,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -314,7 +514,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -366,7 +566,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -425,13 +625,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -440,6 +633,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -504,123 +704,299 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF804328-63E4-4752-9ADB-728D6482BD1F}">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8ACB6CE-280D-4ED1-9FCF-A25BA70014F9}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="97.85546875" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" customWidth="1"/>
-    <col min="4" max="4" width="31" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="27.28515625" customWidth="1"/>
-    <col min="7" max="7" width="27.42578125" customWidth="1"/>
-    <col min="8" max="8" width="28.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="20.42578125" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" customWidth="1"/>
+    <col min="14" max="14" width="16.140625" customWidth="1"/>
+    <col min="15" max="15" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
+      <c r="F3" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="23"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="24"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="12"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="12"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="M8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="O8" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J14" s="3"/>
+    </row>
+    <row r="17" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I17" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="C1:C2"/>
+  <mergeCells count="22">
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="F3:J3"/>
+    <mergeCell ref="F4:J4"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:H9"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="B10:D10"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0" right="0" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>